<commit_message>
visualise-metrics | improve outcome & stream metrics
</commit_message>
<xml_diff>
--- a/steps/visualise-metrics/visualise-metrics.xlsx
+++ b/steps/visualise-metrics/visualise-metrics.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/christracey/workspace/sprint-metrics_webapp/steps/visualise-metrics/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/christracey/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41FB8F27-18D3-E547-BCBA-F73CBBCC9706}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D69664D-6122-CC4C-B4FB-D4EFC515FCDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="68800" windowHeight="28800" tabRatio="783" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="68800" windowHeight="28800" tabRatio="783" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sprint Summary" sheetId="20" r:id="rId1"/>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="159">
   <si>
     <t>Done</t>
   </si>
@@ -572,6 +572,9 @@
     <t>metricConfidence_totalUnestimatedWorkitems</t>
   </si>
   <si>
+    <t>m</t>
+  </si>
+  <si>
     <t>Project1</t>
   </si>
   <si>
@@ -591,7 +594,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -733,25 +736,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Helvetica Neue"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Helvetica Neue"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Helvetica"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="30">
@@ -1247,7 +1231,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="137">
+  <cellXfs count="135">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1450,6 +1434,7 @@
     <xf numFmtId="0" fontId="0" fillId="29" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1522,9 +1507,6 @@
     <xf numFmtId="0" fontId="2" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Input" xfId="1" builtinId="20"/>
@@ -1956,10 +1938,10 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -8249,7 +8231,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="870464" y="2462810"/>
+          <a:off x="889898" y="2482769"/>
           <a:ext cx="2470148" cy="536575"/>
           <a:chOff x="1920877" y="1854200"/>
           <a:chExt cx="2470148" cy="536575"/>
@@ -8413,7 +8395,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="845064" y="5552222"/>
+          <a:off x="864498" y="5579533"/>
           <a:ext cx="2676522" cy="530225"/>
           <a:chOff x="1920877" y="1854200"/>
           <a:chExt cx="2679967" cy="536575"/>
@@ -8615,8 +8597,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="841888" y="8426314"/>
-          <a:ext cx="3241673" cy="753506"/>
+          <a:off x="861322" y="8451525"/>
+          <a:ext cx="3241673" cy="751930"/>
           <a:chOff x="1920876" y="1854200"/>
           <a:chExt cx="3238163" cy="433685"/>
         </a:xfrm>
@@ -9013,7 +8995,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="7946139" y="2472335"/>
+          <a:off x="7963472" y="2492294"/>
           <a:ext cx="2466973" cy="536575"/>
           <a:chOff x="1920877" y="1854200"/>
           <a:chExt cx="2470148" cy="536575"/>
@@ -9181,7 +9163,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="7962014" y="5571272"/>
+          <a:off x="7979347" y="5598583"/>
           <a:ext cx="2355848" cy="530225"/>
           <a:chOff x="1920877" y="1854200"/>
           <a:chExt cx="2340804" cy="536575"/>
@@ -9328,7 +9310,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="8062502" y="6133247"/>
+          <a:off x="8079835" y="6160558"/>
           <a:ext cx="2179786" cy="901700"/>
           <a:chOff x="6190137" y="5534025"/>
           <a:chExt cx="2182604" cy="901700"/>
@@ -9736,7 +9718,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="10771002" y="5549047"/>
+          <a:off x="10789385" y="5576358"/>
           <a:ext cx="2403472" cy="536575"/>
           <a:chOff x="1920877" y="1854200"/>
           <a:chExt cx="2394604" cy="536575"/>
@@ -9966,8 +9948,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="8003288" y="8454889"/>
-          <a:ext cx="3593211" cy="774370"/>
+          <a:off x="8020621" y="8480100"/>
+          <a:ext cx="3594261" cy="772794"/>
           <a:chOff x="1920876" y="1854200"/>
           <a:chExt cx="3354349" cy="441077"/>
         </a:xfrm>
@@ -10113,8 +10095,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="7933437" y="11311194"/>
-          <a:ext cx="3609086" cy="533400"/>
+          <a:off x="7950770" y="11361615"/>
+          <a:ext cx="3610136" cy="533400"/>
           <a:chOff x="1920876" y="1854200"/>
           <a:chExt cx="3354349" cy="536575"/>
         </a:xfrm>
@@ -10260,8 +10242,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="8060438" y="8882415"/>
-          <a:ext cx="4409188" cy="2028924"/>
+          <a:off x="8077771" y="8905525"/>
+          <a:ext cx="4410238" cy="2051509"/>
           <a:chOff x="5203826" y="7785100"/>
           <a:chExt cx="4171950" cy="1466850"/>
         </a:xfrm>
@@ -10386,8 +10368,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="13553631" y="11276269"/>
-          <a:ext cx="6404861" cy="561975"/>
+          <a:off x="13570438" y="11326690"/>
+          <a:ext cx="6387529" cy="561975"/>
           <a:chOff x="1920876" y="1854200"/>
           <a:chExt cx="3354349" cy="536575"/>
         </a:xfrm>
@@ -10588,8 +10570,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="18073253" y="2466352"/>
-          <a:ext cx="1939949" cy="542925"/>
+          <a:off x="18080081" y="2486311"/>
+          <a:ext cx="1932596" cy="542925"/>
           <a:chOff x="1920877" y="1854200"/>
           <a:chExt cx="1808134" cy="536575"/>
         </a:xfrm>
@@ -10735,8 +10717,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="15412067" y="2467083"/>
-          <a:ext cx="2476785" cy="542925"/>
+          <a:off x="15429400" y="2487042"/>
+          <a:ext cx="2476784" cy="542925"/>
           <a:chOff x="2623745" y="1854200"/>
           <a:chExt cx="1815534" cy="536575"/>
         </a:xfrm>
@@ -11026,8 +11008,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="10351996" y="976954"/>
-          <a:ext cx="2703417" cy="536575"/>
+          <a:off x="10369329" y="989034"/>
+          <a:ext cx="2704467" cy="536575"/>
           <a:chOff x="1920877" y="1854200"/>
           <a:chExt cx="2470148" cy="536575"/>
         </a:xfrm>
@@ -11481,8 +11463,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="9501287" y="1867348"/>
-          <a:ext cx="7156934" cy="3283486"/>
+          <a:off x="9518620" y="1879428"/>
+          <a:ext cx="7156934" cy="3291365"/>
           <a:chOff x="8855676" y="1884369"/>
           <a:chExt cx="6442159" cy="3287477"/>
         </a:xfrm>
@@ -11753,7 +11735,7 @@
       <xdr:col>4</xdr:col>
       <xdr:colOff>285845</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>1644525</xdr:rowOff>
+      <xdr:rowOff>1647700</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -11804,9 +11786,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>331304</xdr:colOff>
+      <xdr:colOff>334479</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>1207881</xdr:rowOff>
+      <xdr:rowOff>1211056</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -12478,6 +12460,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="Calibri"/>
             </a:rPr>
+            <a:pPr marL="0" indent="0" algn="l"/>
             <a:t>0</a:t>
           </a:fld>
           <a:endParaRPr lang="en-AU" sz="2000" b="0" i="0" u="none" strike="noStrike">
@@ -13203,7 +13186,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="6041995" y="13145939"/>
+          <a:off x="6061429" y="13196360"/>
           <a:ext cx="880260" cy="240203"/>
           <a:chOff x="5992812" y="13470006"/>
           <a:chExt cx="880260" cy="370395"/>
@@ -13362,7 +13345,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="4976843" y="13373356"/>
+          <a:off x="4996277" y="13423777"/>
           <a:ext cx="1944366" cy="376020"/>
           <a:chOff x="4928706" y="13473112"/>
           <a:chExt cx="1944366" cy="376020"/>
@@ -13591,7 +13574,7 @@
                   <a:cs typeface="Calibri"/>
                 </a:rPr>
                 <a:pPr algn="ctr"/>
-                <a:t>0</a:t>
+                <a:t>#DIV/0!</a:t>
               </a:fld>
               <a:endParaRPr lang="en-AU" sz="800">
                 <a:solidFill>
@@ -13691,7 +13674,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="4976843" y="13730543"/>
+          <a:off x="4996277" y="13780964"/>
           <a:ext cx="1945953" cy="377608"/>
           <a:chOff x="4928706" y="13830299"/>
           <a:chExt cx="1945953" cy="377608"/>
@@ -13848,7 +13831,7 @@
                   <a:cs typeface="Calibri"/>
                 </a:rPr>
                 <a:pPr algn="ctr"/>
-                <a:t>3</a:t>
+                <a:t>0</a:t>
               </a:fld>
               <a:endParaRPr lang="en-AU" sz="800">
                 <a:solidFill>
@@ -13920,7 +13903,7 @@
                   <a:cs typeface="Calibri"/>
                 </a:rPr>
                 <a:pPr algn="ctr"/>
-                <a:t>43</a:t>
+                <a:t>#DIV/0!</a:t>
               </a:fld>
               <a:endParaRPr lang="en-AU" sz="800">
                 <a:solidFill>
@@ -14020,7 +14003,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="4976843" y="14091228"/>
+          <a:off x="4996277" y="14141649"/>
           <a:ext cx="1947033" cy="374110"/>
           <a:chOff x="4928706" y="14190984"/>
           <a:chExt cx="1947033" cy="374110"/>
@@ -14177,7 +14160,7 @@
                   <a:cs typeface="Calibri"/>
                 </a:rPr>
                 <a:pPr algn="ctr"/>
-                <a:t>4</a:t>
+                <a:t>0</a:t>
               </a:fld>
               <a:endParaRPr lang="en-AU" sz="800">
                 <a:solidFill>
@@ -14249,7 +14232,7 @@
                   <a:cs typeface="Calibri"/>
                 </a:rPr>
                 <a:pPr algn="ctr"/>
-                <a:t>57</a:t>
+                <a:t>#DIV/0!</a:t>
               </a:fld>
               <a:endParaRPr lang="en-AU" sz="800">
                 <a:solidFill>
@@ -14349,7 +14332,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="12208116" y="13479963"/>
+          <a:off x="12226499" y="13530384"/>
           <a:ext cx="880260" cy="240203"/>
           <a:chOff x="5992812" y="13470006"/>
           <a:chExt cx="880260" cy="370395"/>
@@ -14508,7 +14491,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="11142964" y="13707380"/>
+          <a:off x="11161347" y="13757801"/>
           <a:ext cx="1944366" cy="376020"/>
           <a:chOff x="4928706" y="13473112"/>
           <a:chExt cx="1944366" cy="376020"/>
@@ -14837,7 +14820,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="11142964" y="14064567"/>
+          <a:off x="11161347" y="14114988"/>
           <a:ext cx="1945953" cy="377608"/>
           <a:chOff x="4928706" y="13830299"/>
           <a:chExt cx="1945953" cy="377608"/>
@@ -15166,7 +15149,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="21198089" y="13114281"/>
+          <a:off x="21197564" y="13164702"/>
           <a:ext cx="880260" cy="240203"/>
           <a:chOff x="5992812" y="13470006"/>
           <a:chExt cx="880260" cy="370395"/>
@@ -15325,7 +15308,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="20132937" y="13341698"/>
+          <a:off x="20132412" y="13392119"/>
           <a:ext cx="1944366" cy="376020"/>
           <a:chOff x="4928706" y="13473112"/>
           <a:chExt cx="1944366" cy="376020"/>
@@ -15654,7 +15637,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="20132937" y="13698885"/>
+          <a:off x="20132412" y="13749306"/>
           <a:ext cx="1945953" cy="377608"/>
           <a:chOff x="4928706" y="13830299"/>
           <a:chExt cx="1945953" cy="377608"/>
@@ -15980,7 +15963,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="20132937" y="14059570"/>
+          <a:off x="20132412" y="14109991"/>
           <a:ext cx="1947033" cy="374110"/>
           <a:chOff x="4928706" y="14190984"/>
           <a:chExt cx="1947033" cy="374110"/>
@@ -16309,8 +16292,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="13550724" y="3429553"/>
-          <a:ext cx="4297827" cy="4272177"/>
+          <a:off x="13567531" y="3449512"/>
+          <a:ext cx="4298352" cy="4279529"/>
           <a:chOff x="12441033" y="3461845"/>
           <a:chExt cx="3993809" cy="4282919"/>
         </a:xfrm>
@@ -17878,8 +17861,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="18269143" y="3426073"/>
-          <a:ext cx="3735039" cy="4327712"/>
+          <a:off x="18275971" y="3446032"/>
+          <a:ext cx="3727686" cy="4335064"/>
           <a:chOff x="16776161" y="3458359"/>
           <a:chExt cx="3601523" cy="4338461"/>
         </a:xfrm>
@@ -19462,22 +19445,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>244230</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>789678</xdr:rowOff>
+      <xdr:colOff>366347</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>769235</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>6773334</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>2862443</xdr:rowOff>
+      <xdr:colOff>5922596</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>2692510</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="207" name="Picture 206">
+        <xdr:cNvPr id="205" name="Picture 204">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F2BCBAB1-65A8-312B-943B-566EE4456888}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{077B5836-BDBA-D653-0F82-DBC6946E668D}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -19485,15 +19468,22 @@
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
-      <xdr:blipFill rotWithShape="1">
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12"/>
-        <a:srcRect t="7678" r="4778"/>
-        <a:stretch/>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1033909" y="3199422"/>
-          <a:ext cx="6529104" cy="2072765"/>
+          <a:off x="1074616" y="6288850"/>
+          <a:ext cx="5556249" cy="1923275"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -19505,22 +19495,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>529166</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>838787</xdr:rowOff>
+      <xdr:colOff>134327</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>751253</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>6567527</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>2682390</xdr:rowOff>
+      <xdr:colOff>6313365</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>2919964</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="209" name="Picture 208">
+        <xdr:cNvPr id="143" name="Picture 142">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{611F218B-C805-B3BE-681A-5C3EB1940EFE}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{917B594D-E5C6-46AF-9D56-E0A17810FA45}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -19529,15 +19519,21 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1318845" y="6333979"/>
-          <a:ext cx="6038361" cy="1843603"/>
+          <a:off x="842596" y="3169138"/>
+          <a:ext cx="6179038" cy="2168711"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -20011,7 +20007,7 @@
   <sheetPr>
     <tabColor rgb="FF006600"/>
   </sheetPr>
-  <dimension ref="B1:M16"/>
+  <dimension ref="B1:R16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8.6640625" style="32" customWidth="1"/>
@@ -20030,8 +20026,8 @@
     <col min="14" max="16384" width="8.6640625" style="32"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:13" ht="42.5" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="2" spans="2:13" ht="10.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="2:18" ht="42.5" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="2:18" ht="10.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="31"/>
       <c r="C2" s="31"/>
       <c r="D2" s="31"/>
@@ -20045,53 +20041,56 @@
       <c r="L2" s="31"/>
       <c r="M2" s="31"/>
     </row>
-    <row r="3" spans="2:13" ht="137" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:18" ht="137" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B3" s="31"/>
-      <c r="C3" s="110"/>
-      <c r="D3" s="111"/>
-      <c r="E3" s="111"/>
-      <c r="F3" s="111"/>
-      <c r="G3" s="111"/>
-      <c r="H3" s="111"/>
-      <c r="I3" s="111"/>
-      <c r="J3" s="111"/>
-      <c r="K3" s="111"/>
-      <c r="L3" s="111"/>
+      <c r="C3" s="111"/>
+      <c r="D3" s="112"/>
+      <c r="E3" s="112"/>
+      <c r="F3" s="112"/>
+      <c r="G3" s="112"/>
+      <c r="H3" s="112"/>
+      <c r="I3" s="112"/>
+      <c r="J3" s="112"/>
+      <c r="K3" s="112"/>
+      <c r="L3" s="112"/>
       <c r="M3" s="36"/>
     </row>
-    <row r="4" spans="2:13" ht="243.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:18" ht="243.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B4" s="31"/>
       <c r="C4" s="29"/>
-      <c r="D4" s="117"/>
-      <c r="E4" s="118"/>
-      <c r="F4" s="124"/>
-      <c r="G4" s="124"/>
-      <c r="H4" s="124"/>
-      <c r="I4" s="125"/>
-      <c r="J4" s="123"/>
-      <c r="K4" s="124"/>
-      <c r="L4" s="125"/>
+      <c r="D4" s="118"/>
+      <c r="E4" s="119"/>
+      <c r="F4" s="125"/>
+      <c r="G4" s="125"/>
+      <c r="H4" s="125"/>
+      <c r="I4" s="126"/>
+      <c r="J4" s="124"/>
+      <c r="K4" s="125"/>
+      <c r="L4" s="126"/>
       <c r="M4" s="31"/>
-    </row>
-    <row r="5" spans="2:13" ht="226.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="R4" s="32" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="5" spans="2:18" ht="226.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B5" s="31"/>
       <c r="C5" s="30"/>
       <c r="D5" s="48"/>
       <c r="E5" s="49"/>
-      <c r="F5" s="112"/>
-      <c r="G5" s="113"/>
-      <c r="H5" s="113"/>
-      <c r="I5" s="114"/>
-      <c r="J5" s="112"/>
-      <c r="K5" s="113"/>
-      <c r="L5" s="114"/>
+      <c r="F5" s="113"/>
+      <c r="G5" s="114"/>
+      <c r="H5" s="114"/>
+      <c r="I5" s="115"/>
+      <c r="J5" s="113"/>
+      <c r="K5" s="114"/>
+      <c r="L5" s="115"/>
       <c r="M5" s="31"/>
     </row>
-    <row r="6" spans="2:13" ht="26.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:18" ht="26.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="31"/>
-      <c r="C6" s="115"/>
-      <c r="D6" s="119"/>
-      <c r="E6" s="120"/>
+      <c r="C6" s="116"/>
+      <c r="D6" s="120"/>
+      <c r="E6" s="121"/>
       <c r="F6" s="35"/>
       <c r="G6" s="37"/>
       <c r="H6" s="38"/>
@@ -20101,29 +20100,29 @@
       <c r="L6" s="39"/>
       <c r="M6" s="31"/>
     </row>
-    <row r="7" spans="2:13" ht="27.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:18" ht="27.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="31"/>
-      <c r="C7" s="116"/>
-      <c r="D7" s="110"/>
-      <c r="E7" s="111"/>
+      <c r="C7" s="117"/>
+      <c r="D7" s="111"/>
+      <c r="E7" s="112"/>
       <c r="F7" s="34"/>
       <c r="G7" s="44"/>
-      <c r="H7" s="126" t="s">
+      <c r="H7" s="127" t="s">
         <v>60</v>
       </c>
-      <c r="I7" s="126"/>
-      <c r="J7" s="126" t="s">
+      <c r="I7" s="127"/>
+      <c r="J7" s="127" t="s">
         <v>61</v>
       </c>
-      <c r="K7" s="126"/>
+      <c r="K7" s="127"/>
       <c r="L7" s="40"/>
       <c r="M7" s="31"/>
     </row>
-    <row r="8" spans="2:13" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:18" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="31"/>
-      <c r="C8" s="116"/>
-      <c r="D8" s="110"/>
-      <c r="E8" s="111"/>
+      <c r="C8" s="117"/>
+      <c r="D8" s="111"/>
+      <c r="E8" s="112"/>
       <c r="F8" s="34"/>
       <c r="G8" s="46" t="s">
         <v>9</v>
@@ -20147,11 +20146,11 @@
       <c r="L8" s="40"/>
       <c r="M8" s="31"/>
     </row>
-    <row r="9" spans="2:13" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:18" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="31"/>
-      <c r="C9" s="116"/>
-      <c r="D9" s="110"/>
-      <c r="E9" s="111"/>
+      <c r="C9" s="117"/>
+      <c r="D9" s="111"/>
+      <c r="E9" s="112"/>
       <c r="F9" s="34"/>
       <c r="G9" s="50" t="s">
         <v>10</v>
@@ -20178,11 +20177,11 @@
       </c>
       <c r="M9" s="31"/>
     </row>
-    <row r="10" spans="2:13" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:18" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="31"/>
-      <c r="C10" s="116"/>
-      <c r="D10" s="110"/>
-      <c r="E10" s="111"/>
+      <c r="C10" s="117"/>
+      <c r="D10" s="111"/>
+      <c r="E10" s="112"/>
       <c r="F10" s="34"/>
       <c r="G10" s="51" t="s">
         <v>56</v>
@@ -20209,11 +20208,11 @@
       </c>
       <c r="M10" s="31"/>
     </row>
-    <row r="11" spans="2:13" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:18" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="31"/>
-      <c r="C11" s="116"/>
-      <c r="D11" s="110"/>
-      <c r="E11" s="111"/>
+      <c r="C11" s="117"/>
+      <c r="D11" s="111"/>
+      <c r="E11" s="112"/>
       <c r="F11" s="34"/>
       <c r="G11" s="46" t="s">
         <v>59</v>
@@ -20237,11 +20236,11 @@
       <c r="L11" s="40"/>
       <c r="M11" s="31"/>
     </row>
-    <row r="12" spans="2:13" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:18" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="31"/>
-      <c r="C12" s="116"/>
-      <c r="D12" s="110"/>
-      <c r="E12" s="111"/>
+      <c r="C12" s="117"/>
+      <c r="D12" s="111"/>
+      <c r="E12" s="112"/>
       <c r="F12" s="34"/>
       <c r="G12" s="46" t="s">
         <v>57</v>
@@ -20265,11 +20264,11 @@
       <c r="L12" s="40"/>
       <c r="M12" s="31"/>
     </row>
-    <row r="13" spans="2:13" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:18" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="31"/>
-      <c r="C13" s="116"/>
-      <c r="D13" s="110"/>
-      <c r="E13" s="111"/>
+      <c r="C13" s="117"/>
+      <c r="D13" s="111"/>
+      <c r="E13" s="112"/>
       <c r="F13" s="34"/>
       <c r="G13" s="46" t="s">
         <v>58</v>
@@ -20293,11 +20292,11 @@
       <c r="L13" s="40"/>
       <c r="M13" s="31"/>
     </row>
-    <row r="14" spans="2:13" ht="42.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:18" ht="42.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B14" s="31"/>
-      <c r="C14" s="116"/>
-      <c r="D14" s="121"/>
-      <c r="E14" s="122"/>
+      <c r="C14" s="117"/>
+      <c r="D14" s="122"/>
+      <c r="E14" s="123"/>
       <c r="F14" s="33"/>
       <c r="G14" s="41"/>
       <c r="H14" s="42"/>
@@ -20307,21 +20306,21 @@
       <c r="L14" s="43"/>
       <c r="M14" s="31"/>
     </row>
-    <row r="15" spans="2:13" ht="264.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:18" ht="264.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B15" s="31"/>
-      <c r="C15" s="116"/>
-      <c r="D15" s="117"/>
-      <c r="E15" s="118"/>
-      <c r="F15" s="112"/>
-      <c r="G15" s="113"/>
-      <c r="H15" s="113"/>
-      <c r="I15" s="113"/>
-      <c r="J15" s="113"/>
-      <c r="K15" s="113"/>
-      <c r="L15" s="114"/>
+      <c r="C15" s="117"/>
+      <c r="D15" s="118"/>
+      <c r="E15" s="119"/>
+      <c r="F15" s="113"/>
+      <c r="G15" s="114"/>
+      <c r="H15" s="114"/>
+      <c r="I15" s="114"/>
+      <c r="J15" s="114"/>
+      <c r="K15" s="114"/>
+      <c r="L15" s="115"/>
       <c r="M15" s="36"/>
     </row>
-    <row r="16" spans="2:13" ht="10" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:18" ht="10" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="31"/>
       <c r="C16" s="31"/>
       <c r="D16" s="31"/>
@@ -20981,7 +20980,7 @@
       </c>
       <c r="B27" s="4">
         <f>SUM(B29:B31)</f>
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="C27" s="4"/>
       <c r="D27" s="4"/>
@@ -21044,9 +21043,9 @@
         <f>'Calculated Stats'!C130</f>
         <v>0</v>
       </c>
-      <c r="C29" s="54">
+      <c r="C29" s="54" t="e">
         <f>ROUND(B29/B$27*100,0)</f>
-        <v>0</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="D29" s="4"/>
       <c r="E29" s="4"/>
@@ -21080,12 +21079,12 @@
         <v>Project1</v>
       </c>
       <c r="B30" s="54">
-        <f>MATCH(A30, 'Calculated Stats'!B$36:B$45, 0)</f>
-        <v>3</v>
-      </c>
-      <c r="C30" s="54">
+        <f>INDEX('Calculated Stats'!D$36:D$45, MATCH(A30, 'Calculated Stats'!B$36:B$45, 0))</f>
+        <v>0</v>
+      </c>
+      <c r="C30" s="54" t="e">
         <f t="shared" ref="C30:C31" si="0">ROUND(B30/B$27*100,0)</f>
-        <v>43</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="D30" s="4"/>
       <c r="E30" s="4"/>
@@ -21112,12 +21111,12 @@
         <v>Project2</v>
       </c>
       <c r="B31" s="54">
-        <f>MATCH(A31, 'Calculated Stats'!B$36:B$45, 0)</f>
-        <v>4</v>
-      </c>
-      <c r="C31" s="54">
+        <f>INDEX('Calculated Stats'!D$36:D$45, MATCH(A31, 'Calculated Stats'!B$36:B$45, 0))</f>
+        <v>0</v>
+      </c>
+      <c r="C31" s="54" t="e">
         <f t="shared" si="0"/>
-        <v>57</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="D31" s="4"/>
       <c r="E31" s="4"/>
@@ -21760,10 +21759,10 @@
       <c r="G5" s="105"/>
     </row>
     <row r="6" spans="2:7" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="127" t="s">
+      <c r="B6" s="128" t="s">
         <v>133</v>
       </c>
-      <c r="C6" s="128"/>
+      <c r="C6" s="129"/>
       <c r="D6" s="105"/>
       <c r="E6" s="105"/>
       <c r="F6" s="106"/>
@@ -21786,7 +21785,7 @@
         <v>1</v>
       </c>
       <c r="C8" s="79" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D8" s="105"/>
       <c r="E8" s="105"/>
@@ -21798,7 +21797,7 @@
         <v>53</v>
       </c>
       <c r="C9" s="79" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D9" s="105"/>
       <c r="E9" s="105"/>
@@ -21807,10 +21806,10 @@
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B10" s="76" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C10" s="79" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D10" s="105"/>
       <c r="E10" s="105"/>
@@ -21819,7 +21818,7 @@
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B11" s="76" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C11" s="79"/>
       <c r="D11" s="105"/>
@@ -22034,10 +22033,10 @@
       <c r="G31" s="105"/>
     </row>
     <row r="32" spans="2:7" ht="27.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B32" s="127" t="s">
+      <c r="B32" s="128" t="s">
         <v>135</v>
       </c>
-      <c r="C32" s="128"/>
+      <c r="C32" s="129"/>
       <c r="D32" s="28"/>
       <c r="E32" s="28"/>
       <c r="F32" s="94"/>
@@ -22056,10 +22055,10 @@
       <c r="B34" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="C34" s="132" t="s">
+      <c r="C34" s="133" t="s">
         <v>5</v>
       </c>
-      <c r="D34" s="132"/>
+      <c r="D34" s="133"/>
       <c r="E34" s="105"/>
       <c r="F34" s="105"/>
       <c r="G34" s="104"/>
@@ -22090,7 +22089,7 @@
         <v>0</v>
       </c>
       <c r="D36" s="4">
-        <f>'processed | data'!B28</f>
+        <f>'processed | data'!B29</f>
         <v>0</v>
       </c>
       <c r="E36" s="105"/>
@@ -22108,7 +22107,7 @@
         <v>0</v>
       </c>
       <c r="D37" s="4">
-        <f>'processed | data'!B29</f>
+        <f>'processed | data'!B30</f>
         <v>0</v>
       </c>
       <c r="E37" s="105"/>
@@ -22126,7 +22125,7 @@
         <v>0</v>
       </c>
       <c r="D38" s="4">
-        <f>'processed | data'!B30</f>
+        <f>'processed | data'!B31</f>
         <v>0</v>
       </c>
       <c r="E38" s="105"/>
@@ -22144,7 +22143,7 @@
         <v>0</v>
       </c>
       <c r="D39" s="4">
-        <f>'processed | data'!B31</f>
+        <f>'processed | data'!B32</f>
         <v>0</v>
       </c>
       <c r="E39" s="105"/>
@@ -22162,7 +22161,7 @@
         <v>0</v>
       </c>
       <c r="D40" s="4">
-        <f>'processed | data'!B32</f>
+        <f>'processed | data'!B33</f>
         <v>0</v>
       </c>
       <c r="E40" s="105"/>
@@ -22180,7 +22179,7 @@
         <v>0</v>
       </c>
       <c r="D41" s="4">
-        <f>'processed | data'!B33</f>
+        <f>'processed | data'!B34</f>
         <v>0</v>
       </c>
       <c r="E41" s="105"/>
@@ -22198,7 +22197,7 @@
         <v>0</v>
       </c>
       <c r="D42" s="4">
-        <f>'processed | data'!B34</f>
+        <f>'processed | data'!B35</f>
         <v>0</v>
       </c>
       <c r="E42" s="105"/>
@@ -22216,7 +22215,7 @@
         <v>0</v>
       </c>
       <c r="D43" s="4">
-        <f>'processed | data'!B35</f>
+        <f>'processed | data'!B36</f>
         <v>0</v>
       </c>
       <c r="E43" s="105"/>
@@ -22234,7 +22233,7 @@
         <v>0</v>
       </c>
       <c r="D44" s="4">
-        <f>'processed | data'!B36</f>
+        <f>'processed | data'!B37</f>
         <v>0</v>
       </c>
       <c r="E44" s="105"/>
@@ -22252,7 +22251,7 @@
         <v>0</v>
       </c>
       <c r="D45" s="4">
-        <f>'processed | data'!B37</f>
+        <f>'processed | data'!B38</f>
         <v>0</v>
       </c>
       <c r="E45" s="105"/>
@@ -22291,10 +22290,10 @@
       <c r="B49" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="C49" s="132" t="s">
+      <c r="C49" s="133" t="s">
         <v>83</v>
       </c>
-      <c r="D49" s="132"/>
+      <c r="D49" s="133"/>
       <c r="E49" s="105"/>
       <c r="F49" s="105"/>
       <c r="G49" s="105"/>
@@ -22526,10 +22525,10 @@
       <c r="B64" s="55" t="s">
         <v>27</v>
       </c>
-      <c r="C64" s="133" t="s">
+      <c r="C64" s="134" t="s">
         <v>5</v>
       </c>
-      <c r="D64" s="133"/>
+      <c r="D64" s="134"/>
       <c r="E64" s="105"/>
       <c r="F64" s="105"/>
       <c r="G64" s="105"/>
@@ -22761,10 +22760,10 @@
       <c r="B79" s="55" t="s">
         <v>27</v>
       </c>
-      <c r="C79" s="133" t="s">
+      <c r="C79" s="134" t="s">
         <v>83</v>
       </c>
-      <c r="D79" s="133"/>
+      <c r="D79" s="134"/>
       <c r="E79" s="105"/>
       <c r="F79" s="105"/>
       <c r="G79" s="105"/>
@@ -23045,7 +23044,7 @@
         <v>0</v>
       </c>
       <c r="D97" s="7">
-        <f>SUM(D36:D37)</f>
+        <f>SUM(D36:D36)</f>
         <v>0</v>
       </c>
       <c r="E97" s="7" t="e">
@@ -23065,7 +23064,7 @@
         <v>0</v>
       </c>
       <c r="D98" s="7">
-        <f>D38</f>
+        <f>D37</f>
         <v>0</v>
       </c>
       <c r="E98" s="7" t="e">
@@ -23085,7 +23084,7 @@
         <v>0</v>
       </c>
       <c r="D99" s="7">
-        <f>D39</f>
+        <f>D38</f>
         <v>0</v>
       </c>
       <c r="E99" s="7" t="e">
@@ -23147,14 +23146,14 @@
     </row>
     <row r="104" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B104" s="6"/>
-      <c r="C104" s="129" t="s">
+      <c r="C104" s="130" t="s">
         <v>6</v>
       </c>
-      <c r="D104" s="130"/>
-      <c r="E104" s="129" t="s">
+      <c r="D104" s="131"/>
+      <c r="E104" s="130" t="s">
         <v>8</v>
       </c>
-      <c r="F104" s="131"/>
+      <c r="F104" s="132"/>
       <c r="G104" s="6"/>
       <c r="N104" s="107"/>
     </row>
@@ -23496,7 +23495,7 @@
         <v>1</v>
       </c>
       <c r="C127" s="101">
-        <f>INDEX( D$36:D$45, MATCH(B127, B$36:B$45,))</f>
+        <f>INDEX( D$36:D$44, MATCH(B127, B$36:B$45,))</f>
         <v>0</v>
       </c>
       <c r="D127" s="101"/>
@@ -23510,7 +23509,7 @@
         <v>53</v>
       </c>
       <c r="C128" s="101">
-        <f>INDEX( D$36:D$45, MATCH(B128, B$36:B$45,))</f>
+        <f>INDEX( D$36:D$44, MATCH(B128, B$36:B$45,))</f>
         <v>0</v>
       </c>
       <c r="D128" s="101"/>
@@ -30093,196 +30092,12 @@
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
-  <dimension ref="A1:CL2"/>
+  <dimension ref="C2:D2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="80" max="80" width="40.1640625" bestFit="1" customWidth="1"/>
-    <col min="81" max="81" width="41.1640625" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:90" x14ac:dyDescent="0.2">
-      <c r="A1" s="135"/>
-      <c r="B1" s="135"/>
-      <c r="C1" s="135"/>
-      <c r="D1" s="135"/>
-      <c r="E1" s="135"/>
-      <c r="F1" s="135"/>
-      <c r="G1" s="135"/>
-      <c r="H1" s="135"/>
-      <c r="I1" s="135"/>
-      <c r="J1" s="135"/>
-      <c r="K1" s="135"/>
-      <c r="L1" s="135"/>
-      <c r="M1" s="135"/>
-      <c r="N1" s="135"/>
-      <c r="O1" s="135"/>
-      <c r="P1" s="135"/>
-      <c r="Q1" s="135"/>
-      <c r="R1" s="135"/>
-      <c r="S1" s="135"/>
-      <c r="T1" s="135"/>
-      <c r="U1" s="135"/>
-      <c r="V1" s="135"/>
-      <c r="W1" s="135"/>
-      <c r="X1" s="135"/>
-      <c r="Y1" s="135"/>
-      <c r="Z1" s="135"/>
-      <c r="AA1" s="135"/>
-      <c r="AB1" s="135"/>
-      <c r="AC1" s="135"/>
-      <c r="AD1" s="135"/>
-      <c r="AE1" s="135"/>
-      <c r="AF1" s="135"/>
-      <c r="AG1" s="135"/>
-      <c r="AH1" s="135"/>
-      <c r="AI1" s="135"/>
-      <c r="AJ1" s="135"/>
-      <c r="AK1" s="135"/>
-      <c r="AL1" s="135"/>
-      <c r="AM1" s="135"/>
-      <c r="AN1" s="135"/>
-      <c r="AO1" s="135"/>
-      <c r="AP1" s="135"/>
-      <c r="AQ1" s="135"/>
-      <c r="AR1" s="135"/>
-      <c r="AS1" s="135"/>
-      <c r="AT1" s="135"/>
-      <c r="AU1" s="135"/>
-      <c r="AV1" s="135"/>
-      <c r="AW1" s="135"/>
-      <c r="AX1" s="135"/>
-      <c r="AY1" s="135"/>
-      <c r="AZ1" s="135"/>
-      <c r="BA1" s="135"/>
-      <c r="BB1" s="135"/>
-      <c r="BC1" s="135"/>
-      <c r="BD1" s="135"/>
-      <c r="BE1" s="135"/>
-      <c r="BF1" s="135"/>
-      <c r="BG1" s="135"/>
-      <c r="BH1" s="135"/>
-      <c r="BI1" s="135"/>
-      <c r="BJ1" s="135"/>
-      <c r="BK1" s="135"/>
-      <c r="BL1" s="135"/>
-      <c r="BM1" s="135"/>
-      <c r="BN1" s="135"/>
-      <c r="BO1" s="135"/>
-      <c r="BP1" s="135"/>
-      <c r="BQ1" s="135"/>
-      <c r="BR1" s="135"/>
-      <c r="BS1" s="135"/>
-      <c r="BT1" s="135"/>
-      <c r="BU1" s="135"/>
-      <c r="BV1" s="135"/>
-      <c r="BW1" s="135"/>
-      <c r="BX1" s="135"/>
-      <c r="BY1" s="135"/>
-      <c r="BZ1" s="135"/>
-      <c r="CA1" s="135"/>
-      <c r="CB1" s="135"/>
-      <c r="CC1" s="135"/>
-      <c r="CD1" s="135"/>
-      <c r="CE1" s="135"/>
-      <c r="CF1" s="135"/>
-      <c r="CG1" s="135"/>
-      <c r="CH1" s="135"/>
-      <c r="CI1" s="135"/>
-      <c r="CJ1" s="135"/>
-      <c r="CK1" s="135"/>
-      <c r="CL1" s="135"/>
-    </row>
-    <row r="2" spans="1:90" ht="16" x14ac:dyDescent="0.2">
-      <c r="A2" s="136"/>
-      <c r="B2" s="136"/>
-      <c r="C2" s="136"/>
-      <c r="D2" s="136"/>
-      <c r="E2" s="134"/>
-      <c r="F2" s="134"/>
-      <c r="G2" s="134"/>
-      <c r="H2" s="134"/>
-      <c r="I2" s="134"/>
-      <c r="J2" s="134"/>
-      <c r="K2" s="136"/>
-      <c r="L2" s="136"/>
-      <c r="M2" s="136"/>
-      <c r="N2" s="136"/>
-      <c r="O2" s="134"/>
-      <c r="P2" s="134"/>
-      <c r="Q2" s="134"/>
-      <c r="R2" s="134"/>
-      <c r="S2" s="134"/>
-      <c r="T2" s="134"/>
-      <c r="U2" s="134"/>
-      <c r="V2" s="134"/>
-      <c r="W2" s="134"/>
-      <c r="X2" s="134"/>
-      <c r="Y2" s="134"/>
-      <c r="Z2" s="134"/>
-      <c r="AA2" s="134"/>
-      <c r="AB2" s="134"/>
-      <c r="AC2" s="134"/>
-      <c r="AD2" s="134"/>
-      <c r="AE2" s="134"/>
-      <c r="AF2" s="134"/>
-      <c r="AG2" s="134"/>
-      <c r="AH2" s="134"/>
-      <c r="AI2" s="134"/>
-      <c r="AJ2" s="134"/>
-      <c r="AK2" s="134"/>
-      <c r="AL2" s="134"/>
-      <c r="AM2" s="134"/>
-      <c r="AN2" s="134"/>
-      <c r="AO2" s="134"/>
-      <c r="AP2" s="134"/>
-      <c r="AQ2" s="134"/>
-      <c r="AR2" s="134"/>
-      <c r="AS2" s="134"/>
-      <c r="AT2" s="134"/>
-      <c r="AU2" s="134"/>
-      <c r="AV2" s="134"/>
-      <c r="AW2" s="134"/>
-      <c r="AX2" s="134"/>
-      <c r="AY2" s="134"/>
-      <c r="AZ2" s="134"/>
-      <c r="BA2" s="134"/>
-      <c r="BB2" s="134"/>
-      <c r="BC2" s="134"/>
-      <c r="BD2" s="134"/>
-      <c r="BE2" s="134"/>
-      <c r="BF2" s="134"/>
-      <c r="BG2" s="134"/>
-      <c r="BH2" s="134"/>
-      <c r="BI2" s="134"/>
-      <c r="BJ2" s="134"/>
-      <c r="BK2" s="134"/>
-      <c r="BL2" s="134"/>
-      <c r="BM2" s="134"/>
-      <c r="BN2" s="134"/>
-      <c r="BO2" s="134"/>
-      <c r="BP2" s="134"/>
-      <c r="BQ2" s="134"/>
-      <c r="BR2" s="134"/>
-      <c r="BS2" s="134"/>
-      <c r="BT2" s="134"/>
-      <c r="BU2" s="134"/>
-      <c r="BV2" s="134"/>
-      <c r="BW2" s="134"/>
-      <c r="BX2" s="134"/>
-      <c r="BY2" s="134"/>
-      <c r="BZ2" s="134"/>
-      <c r="CA2" s="134"/>
-      <c r="CB2" s="134"/>
-      <c r="CC2" s="134"/>
-      <c r="CD2" s="136"/>
-      <c r="CE2" s="136"/>
-      <c r="CF2" s="136"/>
-      <c r="CG2" s="136"/>
-      <c r="CH2" s="136"/>
-      <c r="CI2" s="134"/>
-      <c r="CJ2" s="134"/>
-      <c r="CK2" s="134"/>
-      <c r="CL2" s="134"/>
+    <row r="2" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C2" s="110"/>
+      <c r="D2" s="110"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
visualise-metrics | mark sample images with sample
</commit_message>
<xml_diff>
--- a/steps/visualise-metrics/visualise-metrics.xlsx
+++ b/steps/visualise-metrics/visualise-metrics.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/christracey/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/christracey/workspace/sprint-metrics_webapp/steps/visualise-metrics/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D69664D-6122-CC4C-B4FB-D4EFC515FCDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB4E5D8E-E245-544B-B021-B52E37DFDA98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="68800" windowHeight="28800" tabRatio="783" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="68800" windowHeight="28800" tabRatio="783" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sprint Summary" sheetId="20" r:id="rId1"/>
@@ -19442,7 +19442,131 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>134327</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>751253</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>6313365</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>2919964</xdr:rowOff>
+    </xdr:to>
+    <xdr:grpSp>
+      <xdr:nvGrpSpPr>
+        <xdr:cNvPr id="206" name="Group 205">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D26A9A19-3517-1298-0D23-46C06A8AAB6E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGrpSpPr/>
+      </xdr:nvGrpSpPr>
+      <xdr:grpSpPr>
+        <a:xfrm>
+          <a:off x="932148" y="3160997"/>
+          <a:ext cx="6179038" cy="2168711"/>
+          <a:chOff x="932148" y="3160997"/>
+          <a:chExt cx="6179038" cy="2168711"/>
+        </a:xfrm>
+      </xdr:grpSpPr>
+      <xdr:pic>
+        <xdr:nvPicPr>
+          <xdr:cNvPr id="143" name="Picture 142">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{917B594D-E5C6-46AF-9D56-E0A17810FA45}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvPicPr>
+            <a:picLocks noChangeAspect="1"/>
+          </xdr:cNvPicPr>
+        </xdr:nvPicPr>
+        <xdr:blipFill>
+          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12" cstate="print">
+            <a:extLst>
+              <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+                <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+              </a:ext>
+            </a:extLst>
+          </a:blip>
+          <a:stretch>
+            <a:fillRect/>
+          </a:stretch>
+        </xdr:blipFill>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="932148" y="3160997"/>
+            <a:ext cx="6179038" cy="2168711"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+        </xdr:spPr>
+      </xdr:pic>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="55" name="TextBox 54">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D9CE4244-6ED7-4C8B-F82D-B716F6214069}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr txBox="1"/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm rot="821982">
+            <a:off x="3663460" y="3614614"/>
+            <a:ext cx="3337821" cy="797820"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln w="9525" cmpd="sng">
+            <a:noFill/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="dk1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:r>
+              <a:rPr lang="en-GB" sz="6600">
+                <a:solidFill>
+                  <a:srgbClr val="EA9191"/>
+                </a:solidFill>
+                <a:latin typeface="Stencil" pitchFamily="82" charset="77"/>
+              </a:rPr>
+              <a:t>SAMPLE</a:t>
+            </a:r>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+    </xdr:grpSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>366347</xdr:colOff>
@@ -19455,91 +19579,115 @@
       <xdr:row>4</xdr:row>
       <xdr:rowOff>2692510</xdr:rowOff>
     </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="205" name="Picture 204">
+    <xdr:grpSp>
+      <xdr:nvGrpSpPr>
+        <xdr:cNvPr id="207" name="Group 206">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{077B5836-BDBA-D653-0F82-DBC6946E668D}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{25B12F7D-8CAE-6F07-AF74-5BF5F58E2ABB}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
+        <xdr:cNvGrpSpPr/>
+      </xdr:nvGrpSpPr>
+      <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="1074616" y="6288850"/>
+          <a:off x="1164168" y="6272568"/>
           <a:ext cx="5556249" cy="1923275"/>
+          <a:chOff x="1164168" y="6272568"/>
+          <a:chExt cx="5556249" cy="1923275"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>134327</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>751253</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>6313365</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>2919964</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="143" name="Picture 142">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{917B594D-E5C6-46AF-9D56-E0A17810FA45}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="842596" y="3169138"/>
-          <a:ext cx="6179038" cy="2168711"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
+      </xdr:grpSpPr>
+      <xdr:pic>
+        <xdr:nvPicPr>
+          <xdr:cNvPr id="205" name="Picture 204">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{077B5836-BDBA-D653-0F82-DBC6946E668D}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvPicPr>
+            <a:picLocks noChangeAspect="1"/>
+          </xdr:cNvPicPr>
+        </xdr:nvPicPr>
+        <xdr:blipFill>
+          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13" cstate="print">
+            <a:extLst>
+              <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+                <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+              </a:ext>
+            </a:extLst>
+          </a:blip>
+          <a:stretch>
+            <a:fillRect/>
+          </a:stretch>
+        </xdr:blipFill>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="1164168" y="6272568"/>
+            <a:ext cx="5556249" cy="1923275"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+        </xdr:spPr>
+      </xdr:pic>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="113" name="TextBox 112">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9937D27D-D992-F946-9EFF-5677DB74CBF7}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr txBox="1"/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm rot="20758441">
+            <a:off x="2350476" y="6746631"/>
+            <a:ext cx="3337821" cy="797820"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln w="9525" cmpd="sng">
+            <a:noFill/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="dk1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:r>
+              <a:rPr lang="en-GB" sz="6600">
+                <a:solidFill>
+                  <a:srgbClr val="EA9191"/>
+                </a:solidFill>
+                <a:latin typeface="Stencil" pitchFamily="82" charset="77"/>
+              </a:rPr>
+              <a:t>SAMPLE</a:t>
+            </a:r>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+    </xdr:grpSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>

</xml_diff>